<commit_message>
[~] Compose: Valkey instead of Redis
The cache now runs valkey/valkey:9.1.2 (BSD-3-Clause) instead of
redis:7, which had moved to Redis 7.4 under RSALv2 or SSPL. The service
keeps its name and the REDIS_* settings, the healthcheck uses
valkey-cli, and the server starts as valkey-server so it drops root.
Valkey refuses the RDB files Redis 7.4 wrote, so it starts on a new
valkey_data volume; it only held keys that expire within a day.
Checked on a throwaway stack: login, a protected route, logout and the
refused token after it all go through Valkey. Docs, THIRD_PARTY_NOTICES
and the licence inventory follow.
</commit_message>
<xml_diff>
--- a/docs/eip/dependency-licence-inventory.xlsx
+++ b/docs/eip/dependency-licence-inventory.xlsx
@@ -84,7 +84,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -154,6 +154,11 @@
         <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -189,7 +194,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -312,6 +317,9 @@
       <alignment horizontal="general" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1060,7 +1068,7 @@
     <row r="18" ht="15" customHeight="1" s="21">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>2. Replace the Redis image with Valkey (BSD-3-Clause) or pin redis:7.2; keep RedisInsight out of customer builds.</t>
+          <t>2. ✅ Redis image replaced by Valkey 9.1.2 (BSD-3-Clause) on 07/10; keep RedisInsight out of customer builds.</t>
         </is>
       </c>
     </row>
@@ -62480,42 +62488,42 @@
     <row r="7" ht="46.25" customHeight="1" s="21">
       <c r="A7" s="31" t="inlineStr">
         <is>
-          <t>Redis</t>
+          <t>Valkey</t>
         </is>
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
-          <t>redis:7 (floats to 7.4.x)</t>
+          <t>valkey/valkey:9.1.2</t>
         </is>
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>Cache</t>
+          <t>Cache (Compose service redis)</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Separate container</t>
+          <t>Separate container, unmodified</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>RSALv2 or SSPLv1 (Redis 7.4+). 7.2 and earlier: BSD-3-Clause</t>
-        </is>
-      </c>
-      <c r="F7" s="38" t="inlineStr">
-        <is>
-          <t>Source-available</t>
-        </is>
-      </c>
-      <c r="G7" s="38" t="inlineStr">
-        <is>
-          <t>Replace (recommended)</t>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="F7" s="42" t="inlineStr">
+        <is>
+          <t>Permissive</t>
+        </is>
+      </c>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
         <is>
-          <t>RSALv2 lets us use Redis inside Horus (it forbids offering Redis itself as a service). But it is not open source, enterprise legal reviews flag it, and a floating tag can change licence silently. Switch to Valkey (valkey/valkey, BSD-3-Clause, Redis-compatible – redis-py works unchanged) or pin redis:7.2.</t>
+          <t>Keep notice. Replaced redis:7 (Redis 7.4, RSALv2 or SSPLv1) on 07/10/2026; same protocol, redis-py unchanged.</t>
         </is>
       </c>
     </row>
@@ -63721,9 +63729,9 @@
       <c r="A3" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="B3" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C3" s="25" t="inlineStr">
@@ -63748,7 +63756,7 @@
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>Switch to Valkey (BSD-3-Clause, drop-in, redis-py unchanged) or pin redis:7.2.</t>
+          <t>Replaced by valkey/valkey:9.1.2 (BSD-3-Clause); service name and REDIS_* settings unchanged.</t>
         </is>
       </c>
       <c r="H3" s="31" t="inlineStr">
@@ -63758,7 +63766,7 @@
       </c>
       <c r="I3" s="31" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done (07/10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[~] Compose: RedisInsight and PgAdmin only in the dev-tools profile
The two development tools move from the Compose profile admin to
dev-tools: PgAdmin ships with default credentials and RedisInsight has
no login, so neither belongs in a tester's or customer's stack. The
installer never starts that profile; its --admin-profile flag, which
only made their ports required, is gone, and so are their port checks.
A wiring test fails if the installer, the desktop app or the bundle
scripts ever name the profile or COMPOSE_PROFILES. .env.example no
longer advertises a Metabase that does not exist or a RedisInsight
connection that is not set up.
</commit_message>
<xml_diff>
--- a/docs/eip/dependency-licence-inventory.xlsx
+++ b/docs/eip/dependency-licence-inventory.xlsx
@@ -1068,7 +1068,7 @@
     <row r="18" ht="15" customHeight="1" s="21">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>2. ✅ Redis image replaced by Valkey 9.1.2 (BSD-3-Clause) on 07/10; keep RedisInsight out of customer builds.</t>
+          <t>2. ✅ Redis image replaced by Valkey 9.1.2 (BSD-3-Clause) on 07/10; RedisInsight and pgAdmin only in the dev-tools profile, which the installer never starts.</t>
         </is>
       </c>
     </row>
@@ -62540,7 +62540,7 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>DB admin UI (admin profile)</t>
+          <t>DB admin UI (dev-tools profile)</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
@@ -62565,7 +62565,7 @@
       </c>
       <c r="H8" s="25" t="inlineStr">
         <is>
-          <t>Licence OK. Keep it out of the customer profile anyway (admin UI with default credentials).</t>
+          <t>Licence OK. Development tool only: Compose profile dev-tools, which the installer never starts (admin UI with default credentials).</t>
         </is>
       </c>
     </row>
@@ -62582,7 +62582,7 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Cache admin UI (admin profile)</t>
+          <t>Cache admin UI (dev-tools profile)</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
@@ -62607,7 +62607,7 @@
       </c>
       <c r="H9" s="25" t="inlineStr">
         <is>
-          <t>Team/debug tool only. Exclude from the customer bundle.</t>
+          <t>Team/debug tool only: Compose profile dev-tools, which the installer never starts, so it is not in a customer install.</t>
         </is>
       </c>
     </row>
@@ -63774,9 +63774,9 @@
       <c r="A4" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C4" s="25" t="inlineStr">
@@ -63786,7 +63786,7 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>src/infra/docker-compose.yml (admin profile)</t>
+          <t>src/infra/docker-compose.yml (dev-tools profile)</t>
         </is>
       </c>
       <c r="E4" s="25" t="inlineStr">
@@ -63801,7 +63801,7 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>Exclude from the customer bundle; keep for the team only.</t>
+          <t>RedisInsight and pgAdmin moved to the Compose profile dev-tools; the installer never starts it and no longer checks their ports.</t>
         </is>
       </c>
       <c r="H4" s="31" t="inlineStr">
@@ -63811,7 +63811,7 @@
       </c>
       <c r="I4" s="31" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done (07/10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[~] Images: pin every tag
postgres, pgadmin4, redisinsight and prometheus ran on latest, and the
Python and Node base images on minor tags. Each is now pinned to the
exact version its floating tag gives today, checked by digest:
postgres:18.6, dpage/pgadmin4:9.18.0, redis/redisinsight:3.8.0,
prom/prometheus:v3.15.0, python:3.11.17-slim and node:20.20.2-alpine.
A wiring test fails on latest or a tag without an exact version in the
Compose files and Dockerfiles. THIRD_PARTY_NOTICES, the licence
inventory and the version table of architecture.md follow.
</commit_message>
<xml_diff>
--- a/docs/eip/dependency-licence-inventory.xlsx
+++ b/docs/eip/dependency-licence-inventory.xlsx
@@ -775,7 +775,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="21">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -790,7 +789,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="23.85" customHeight="1" s="21">
       <c r="A7" s="26" t="inlineStr">
         <is>
@@ -1050,7 +1048,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="24" t="inlineStr">
         <is>
@@ -1093,7 +1090,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="21">
       <c r="A23" s="24" t="inlineStr">
         <is>
@@ -62451,7 +62447,7 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>postgres:latest</t>
+          <t>postgres:18.6</t>
         </is>
       </c>
       <c r="C6" s="25" t="inlineStr">
@@ -62481,7 +62477,7 @@
       </c>
       <c r="H6" s="25" t="inlineStr">
         <is>
-          <t>Pin a major version instead of latest.</t>
+          <t>Pinned to 18.6, the version latest gave on 07/10/2026.</t>
         </is>
       </c>
     </row>
@@ -62535,7 +62531,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>dpage/pgadmin4:latest</t>
+          <t>dpage/pgadmin4:9.18.0</t>
         </is>
       </c>
       <c r="C8" s="25" t="inlineStr">
@@ -62577,7 +62573,7 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>redis/redisinsight:latest</t>
+          <t>redis/redisinsight:3.8.0</t>
         </is>
       </c>
       <c r="C9" s="25" t="inlineStr">
@@ -62745,7 +62741,7 @@
       </c>
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>prom/prometheus:latest</t>
+          <t>prom/prometheus:v3.15.0</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
@@ -62775,7 +62771,7 @@
       </c>
       <c r="H13" s="25" t="inlineStr">
         <is>
-          <t>Pin a version instead of latest.</t>
+          <t>Pinned to v3.15.0, the version latest gave on 07/10/2026.</t>
         </is>
       </c>
     </row>
@@ -62787,7 +62783,7 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>python:3.11-slim (Debian)</t>
+          <t>python:3.11.17-slim (Debian)</t>
         </is>
       </c>
       <c r="C14" s="25" t="inlineStr">
@@ -62829,7 +62825,7 @@
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>node:20-alpine</t>
+          <t>node:20.20.2-alpine</t>
         </is>
       </c>
       <c r="C15" s="25" t="inlineStr">

</xml_diff>

<commit_message>
[+] CI: fail on a copyleft licence in our own processes
A new ci.yml job, licences, tests the licence scripts, runs
third_party_notices.py --check, then scripts/licences/check_licences.py,
which fails on GPL, AGPL or SSPL among the Python packages, the web
client's production dependencies and the desktop app's crates. An OR
licence passes when one choice is permissive; LGPL is a warning.
Images and models run as separate processes and are only listed.
Reviewed exceptions live in scripts/licences/allowlist.yaml with their
reason; today it holds psycopg2-binary and the sharp/libvips packages
(both LGPL, used unmodified). An entry that no longer matches fails.
</commit_message>
<xml_diff>
--- a/docs/eip/dependency-licence-inventory.xlsx
+++ b/docs/eip/dependency-licence-inventory.xlsx
@@ -775,6 +775,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="21">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -789,6 +790,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="23.85" customHeight="1" s="21">
       <c r="A7" s="26" t="inlineStr">
         <is>
@@ -1048,6 +1050,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="24" t="inlineStr">
         <is>
@@ -1079,7 +1082,7 @@
     <row r="20" ht="15" customHeight="1" s="21">
       <c r="A20" s="29" t="inlineStr">
         <is>
-          <t>4. Pin versions + add a CI licence gate (fail on AGPL/GPL/SSPL inside our processes).</t>
+          <t>4. ✅ Lock files with hashes, pinned image tags and the CI licence gate (job licences, 07/10).</t>
         </is>
       </c>
     </row>
@@ -1090,6 +1093,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="21">
       <c r="A23" s="24" t="inlineStr">
         <is>
@@ -63860,9 +63864,9 @@
       <c r="A6" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C6" s="25" t="inlineStr">
@@ -63887,7 +63891,7 @@
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>Pin versions (uv pip compile → lock files), pin image tags, and add a CI licence gate that fails on AGPL/GPL/SSPL inside our processes.</t>
+          <t>requirements*.lock with hashes for every service, every image tag pinned, and the CI job licences: THIRD_PARTY_NOTICES --check, and it fails on GPL/AGPL/SSPL in our own processes (exceptions in scripts/licences/allowlist.yaml).</t>
         </is>
       </c>
       <c r="H6" s="31" t="inlineStr">
@@ -63897,7 +63901,7 @@
       </c>
       <c r="I6" s="31" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done (07/10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[#] Inventory: GPL source offer, MAS build tools and test tools done
The dependency licence inventory now records what f3bb793 and 9a00c78
did. Flags 7 (poppler-utils) and 12 (test tools in production images)
are done. The base images and poppler-utils point to the written offer
in THIRD_PARTY_NOTICES section 7 and to fetch-gpl-sources.py. The
build-essential / g++ row says the compilers stay in the MAS builder
stage and are no longer shipped. Snapshot date 08/10/2026.
</commit_message>
<xml_diff>
--- a/docs/eip/dependency-licence-inventory.xlsx
+++ b/docs/eip/dependency-licence-inventory.xlsx
@@ -771,11 +771,10 @@
     <row r="2" ht="15" customHeight="1" s="21">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Snapshot 24/09/2026, updated 07/10/2026 · prepared for ADR-004 (closed-source licence)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Snapshot 24/09/2026, updated 08/10/2026 · prepared for ADR-004 (closed-source licence)</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="15" customHeight="1" s="21">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -790,7 +789,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="23.85" customHeight="1" s="21">
       <c r="A7" s="26" t="inlineStr">
         <is>
@@ -1050,7 +1048,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="24" t="inlineStr">
         <is>
@@ -1093,7 +1090,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="21">
       <c r="A23" s="24" t="inlineStr">
         <is>
@@ -62817,7 +62813,7 @@
       </c>
       <c r="H14" s="25" t="inlineStr">
         <is>
-          <t>Normal OS aggregation.</t>
+          <t>Normal OS aggregation. Its GPL and LGPL packages are listed, with the written offer for their source, in THIRD_PARTY_NOTICES section 7 (08/10).</t>
         </is>
       </c>
     </row>
@@ -62859,7 +62855,7 @@
       </c>
       <c r="H15" s="25" t="inlineStr">
         <is>
-          <t>Normal OS aggregation.</t>
+          <t>Normal OS aggregation. Its GPL and LGPL packages are listed, with the written offer for their source, in THIRD_PARTY_NOTICES section 7 (08/10).</t>
         </is>
       </c>
     </row>
@@ -62901,7 +62897,7 @@
       </c>
       <c r="H16" s="25" t="inlineStr">
         <is>
-          <t>Separate program = aggregation, Horus code unaffected. Ship the GPL text + source offer, or replace pdf2image+poppler with pypdfium2 (already installed, Apache-2.0/BSD).</t>
+          <t>Separate program = aggregation, Horus code unaffected. GPL texts in LICENSES/, written offer in THIRD_PARTY_NOTICES section 7, sources gathered by scripts/licences/fetch-gpl-sources.py (08/10). Replacing pdf2image+poppler with pypdfium2 would also remove GnuPG, which poppler pulls in.</t>
         </is>
       </c>
     </row>
@@ -62955,17 +62951,17 @@
       </c>
       <c r="B18" s="31" t="inlineStr">
         <is>
-          <t>Debian packages in mas image</t>
+          <t>Debian packages in the mas builder stage</t>
         </is>
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>Compilers left in the final image</t>
+          <t>Compilers of the build stage, not shipped</t>
         </is>
       </c>
       <c r="D18" s="25" t="inlineStr">
         <is>
-          <t>Build tools (single-stage Dockerfile)</t>
+          <t>Build tools (builder stage of a multi-stage Dockerfile)</t>
         </is>
       </c>
       <c r="E18" s="25" t="inlineStr">
@@ -62978,14 +62974,14 @@
           <t>Strong copyleft</t>
         </is>
       </c>
-      <c r="G18" s="33" t="inlineStr">
-        <is>
-          <t>OK – conditions</t>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H18" s="25" t="inlineStr">
         <is>
-          <t>Runtime-library exception covers compiled output. Better: multi-stage build so compilers are not shipped (smaller, fewer licences to declare).</t>
+          <t>Not in the image since 08/10: the MAS Dockerfile is multi-stage and its final stage installs no system package.</t>
         </is>
       </c>
     </row>
@@ -63954,9 +63950,9 @@
       <c r="A8" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C8" s="25" t="inlineStr">
@@ -63981,7 +63977,7 @@
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>Keep as separate process + notice, or replace pdf2image with pypdfium2 rendering (removes GPL from the image).</t>
+          <t>Kept as a separate process. GPL texts in LICENSES/, written offer in THIRD_PARTY_NOTICES section 7, sources gathered by scripts/licences/fetch-gpl-sources.py. Replacing pdf2image with pypdfium2 rendering would remove it.</t>
         </is>
       </c>
       <c r="H8" s="31" t="inlineStr">
@@ -63991,7 +63987,7 @@
       </c>
       <c r="I8" s="31" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Done (08/10)</t>
         </is>
       </c>
     </row>
@@ -64179,9 +64175,9 @@
       <c r="A13" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="32" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
@@ -64206,7 +64202,7 @@
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>Move to requirements-dev.txt.</t>
+          <t>Moved to requirements-test.txt in each service, which only CI installs; no lock file names a test tool.</t>
         </is>
       </c>
       <c r="H13" s="31" t="inlineStr">
@@ -64216,7 +64212,7 @@
       </c>
       <c r="I13" s="31" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Done (08/10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[-] Compose: remove RedisInsight (SSPL, unused)
RedisInsight was licensed under SSPL-1.0, ran only in the dev-tools
profile, and its connection to Valkey was never set up. The service,
its port 5540 and its volume are gone from the Compose file, and its
note from .env.example. valkey-cli inside the redis container does the
same job: docs/operations.md gives the one command that opens it with
the password the container reads from .env, through VALKEYCLI_AUTH, so
the password stays off the command line (checked on a throwaway Valkey
9.1.2). PgAdmin stays in dev-tools.

README, getting-started, operations, components.yaml,
THIRD_PARTY_NOTICES and the licence inventory follow. LICENSES/SSPL-1.0.txt
goes too, since no component uses that licence any more. tests/ci keeps
the dev-tools check for PgAdmin and fails if RedisInsight comes back.
</commit_message>
<xml_diff>
--- a/docs/eip/dependency-licence-inventory.xlsx
+++ b/docs/eip/dependency-licence-inventory.xlsx
@@ -525,8 +525,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Services" displayName="Services" ref="A1:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:H18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Services" displayName="Services" ref="A1:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:H17"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Component"/>
     <tableColumn id="2" name="Image / package"/>
@@ -775,6 +775,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="21">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -789,6 +790,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="23.85" customHeight="1" s="21">
       <c r="A7" s="26" t="inlineStr">
         <is>
@@ -943,23 +945,23 @@
         </is>
       </c>
       <c r="B11" s="27">
-        <f>COUNTIF('Services &amp; images'!$F$2:$F$18,"Permissive")</f>
+        <f>COUNTIF('Services &amp; images'!$F$2:$F$17,"Permissive")</f>
         <v/>
       </c>
       <c r="C11" s="27">
-        <f>COUNTIF('Services &amp; images'!$F$2:$F$18,"Weak copyleft")</f>
+        <f>COUNTIF('Services &amp; images'!$F$2:$F$17,"Weak copyleft")</f>
         <v/>
       </c>
       <c r="D11" s="27">
-        <f>COUNTIF('Services &amp; images'!$F$2:$F$18,"Strong copyleft")</f>
+        <f>COUNTIF('Services &amp; images'!$F$2:$F$17,"Strong copyleft")</f>
         <v/>
       </c>
       <c r="E11" s="27">
-        <f>COUNTIF('Services &amp; images'!$F$2:$F$18,"Source-available")</f>
+        <f>COUNTIF('Services &amp; images'!$F$2:$F$17,"Source-available")</f>
         <v/>
       </c>
       <c r="F11" s="27">
-        <f>COUNTIF('Services &amp; images'!$F$2:$F$18,"Third-party proprietary")</f>
+        <f>COUNTIF('Services &amp; images'!$F$2:$F$17,"Third-party proprietary")</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -967,7 +969,7 @@
         <v/>
       </c>
       <c r="H11" s="28">
-        <f>COUNTIF('Services &amp; images'!$G$2:$G$18,"Blocker*")</f>
+        <f>COUNTIF('Services &amp; images'!$G$2:$G$17,"Blocker*")</f>
         <v/>
       </c>
     </row>
@@ -1048,6 +1050,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="24" t="inlineStr">
         <is>
@@ -1065,7 +1068,7 @@
     <row r="18" ht="15" customHeight="1" s="21">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>2. ✅ Redis image replaced by Valkey 9.1.2 (BSD-3-Clause) on 07/10; RedisInsight and pgAdmin only in the dev-tools profile, which the installer never starts.</t>
+          <t>2. ✅ Redis image replaced by Valkey 9.1.2 (BSD-3-Clause) on 07/10; RedisInsight (SSPL) removed on 08/10; pgAdmin only in the dev-tools profile, which the installer never starts.</t>
         </is>
       </c>
     </row>
@@ -1090,6 +1093,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="21">
       <c r="A23" s="24" t="inlineStr">
         <is>
@@ -62216,7 +62220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="20" min="1" max="1"/>
@@ -62565,67 +62569,67 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="21">
+    <row r="9" ht="35.05" customHeight="1" s="21">
       <c r="A9" s="31" t="inlineStr">
         <is>
-          <t>RedisInsight</t>
+          <t>Grafana Loki</t>
         </is>
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>redis/redisinsight:3.8.0</t>
+          <t>grafana/loki:3.4.2</t>
         </is>
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Cache admin UI (dev-tools profile)</t>
+          <t>Log storage (/admin/logs)</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>Separate container</t>
+          <t>Separate container, unmodified, HTTP API only</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>SSPL-1.0</t>
+          <t>AGPL-3.0-only</t>
         </is>
       </c>
       <c r="F9" s="38" t="inlineStr">
         <is>
-          <t>Source-available</t>
-        </is>
-      </c>
-      <c r="G9" s="38" t="inlineStr">
-        <is>
-          <t>Do not ship to customers</t>
+          <t>Strong copyleft</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>OK – conditions</t>
         </is>
       </c>
       <c r="H9" s="25" t="inlineStr">
         <is>
-          <t>Team/debug tool only: Compose profile dev-tools, which the installer never starts, so it is not in a customer install.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="35.05" customHeight="1" s="21">
+          <t>Does not make Horus AGPL: it is a separate program we talk to over HTTP. Conditions: never modify or fork it; ship the AGPL text + link to the exact upstream source. If a customer's policy bans AGPL, swap for an Apache-licensed store.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="23.85" customHeight="1" s="21">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>Grafana Loki</t>
+          <t>Grafana Tempo</t>
         </is>
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>grafana/loki:3.4.2</t>
+          <t>grafana/tempo:2.6.0</t>
         </is>
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Log storage (/admin/logs)</t>
+          <t>Traces (/admin/traces)</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>Separate container, unmodified, HTTP API only</t>
+          <t>Separate container, unmodified, HTTP/OTLP</t>
         </is>
       </c>
       <c r="E10" s="25" t="inlineStr">
@@ -62645,71 +62649,71 @@
       </c>
       <c r="H10" s="25" t="inlineStr">
         <is>
-          <t>Does not make Horus AGPL: it is a separate program we talk to over HTTP. Conditions: never modify or fork it; ship the AGPL text + link to the exact upstream source. If a customer's policy bans AGPL, swap for an Apache-licensed store.</t>
+          <t>Same as Loki. Alternative if needed: Jaeger (Apache-2.0).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="23.85" customHeight="1" s="21">
       <c r="A11" s="31" t="inlineStr">
         <is>
-          <t>Grafana Tempo</t>
+          <t>Grafana Alloy</t>
         </is>
       </c>
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>grafana/tempo:2.6.0</t>
+          <t>grafana/alloy:v1.20.1</t>
         </is>
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>Traces (/admin/traces)</t>
+          <t>Ships container logs to Loki</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>Separate container, unmodified, HTTP/OTLP</t>
+          <t>Separate container, reads the Docker socket read-only</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>AGPL-3.0-only</t>
-        </is>
-      </c>
-      <c r="F11" s="38" t="inlineStr">
-        <is>
-          <t>Strong copyleft</t>
-        </is>
-      </c>
-      <c r="G11" s="33" t="inlineStr">
-        <is>
-          <t>OK – conditions</t>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>Permissive</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H11" s="25" t="inlineStr">
         <is>
-          <t>Same as Loki. Alternative if needed: Jaeger (Apache-2.0).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="23.85" customHeight="1" s="21">
+          <t>Replaced Promtail (end of life since March 2026) on 08/10/2026, with the same Loki labels for /admin/logs. Pinned to v1.20.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="21">
       <c r="A12" s="31" t="inlineStr">
         <is>
-          <t>Grafana Alloy</t>
+          <t>Prometheus</t>
         </is>
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
-          <t>grafana/alloy:v1.20.1</t>
+          <t>prom/prometheus:v3.15.0</t>
         </is>
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Ships container logs to Loki</t>
+          <t>Metrics (/admin/metrics)</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>Separate container, reads the Docker socket read-only</t>
+          <t>Separate container</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr">
@@ -62729,34 +62733,34 @@
       </c>
       <c r="H12" s="25" t="inlineStr">
         <is>
-          <t>Replaced Promtail (end of life since March 2026) on 08/10/2026, with the same Loki labels for /admin/logs. Pinned to v1.20.1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="21">
+          <t>Pinned to v3.15.0, the version latest gave on 07/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="23.85" customHeight="1" s="21">
       <c r="A13" s="31" t="inlineStr">
         <is>
-          <t>Prometheus</t>
+          <t>Python base image</t>
         </is>
       </c>
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>prom/prometheus:v3.15.0</t>
+          <t>python:3.11.17-slim (Debian)</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>Metrics (/admin/metrics)</t>
+          <t>Base of mas, agent, knowledge-store</t>
         </is>
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
-          <t>Separate container</t>
+          <t>OS layer</t>
         </is>
       </c>
       <c r="E13" s="25" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>PSF-2.0 (Python) + Debian packages (mixed)</t>
         </is>
       </c>
       <c r="F13" s="32" t="inlineStr">
@@ -62771,24 +62775,24 @@
       </c>
       <c r="H13" s="25" t="inlineStr">
         <is>
-          <t>Pinned to v3.15.0, the version latest gave on 07/10/2026.</t>
+          <t>Normal OS aggregation. Its GPL and LGPL packages are listed, with the written offer for their source, in THIRD_PARTY_NOTICES section 7 (08/10).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" s="21">
       <c r="A14" s="31" t="inlineStr">
         <is>
-          <t>Python base image</t>
+          <t>Node base image</t>
         </is>
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>python:3.11.17-slim (Debian)</t>
+          <t>node:20.20.2-alpine</t>
         </is>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>Base of mas, agent, knowledge-store</t>
+          <t>Base of web-client</t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
@@ -62798,7 +62802,7 @@
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>PSF-2.0 (Python) + Debian packages (mixed)</t>
+          <t>MIT (Node.js) + Alpine packages (mixed)</t>
         </is>
       </c>
       <c r="F14" s="32" t="inlineStr">
@@ -62820,49 +62824,49 @@
     <row r="15" ht="23.85" customHeight="1" s="21">
       <c r="A15" s="31" t="inlineStr">
         <is>
-          <t>Node base image</t>
+          <t>poppler-utils</t>
         </is>
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>node:20.20.2-alpine</t>
+          <t>Debian package in knowledge-store image</t>
         </is>
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Base of web-client</t>
+          <t>PDF → image (called by pdf2image)</t>
         </is>
       </c>
       <c r="D15" s="25" t="inlineStr">
         <is>
-          <t>OS layer</t>
+          <t>Separate program (pdftoppm), not linked</t>
         </is>
       </c>
       <c r="E15" s="25" t="inlineStr">
         <is>
-          <t>MIT (Node.js) + Alpine packages (mixed)</t>
-        </is>
-      </c>
-      <c r="F15" s="32" t="inlineStr">
-        <is>
-          <t>Permissive</t>
-        </is>
-      </c>
-      <c r="G15" s="32" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>GPL-2.0 or GPL-3.0</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>Strong copyleft</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>OK – conditions</t>
         </is>
       </c>
       <c r="H15" s="25" t="inlineStr">
         <is>
-          <t>Normal OS aggregation. Its GPL and LGPL packages are listed, with the written offer for their source, in THIRD_PARTY_NOTICES section 7 (08/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="23.85" customHeight="1" s="21">
+          <t>Separate program = aggregation, Horus code unaffected. GPL texts in LICENSES/, written offer in THIRD_PARTY_NOTICES section 7, sources gathered by scripts/licences/fetch-gpl-sources.py (08/10). Replacing pdf2image+poppler with pypdfium2 would also remove GnuPG, which poppler pulls in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="31" t="inlineStr">
         <is>
-          <t>poppler-utils</t>
+          <t>tesseract-ocr</t>
         </is>
       </c>
       <c r="B16" s="31" t="inlineStr">
@@ -62872,119 +62876,78 @@
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
-          <t>PDF → image (called by pdf2image)</t>
+          <t>OCR</t>
         </is>
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
-          <t>Separate program (pdftoppm), not linked</t>
+          <t>Separate program via pytesseract</t>
         </is>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
-          <t>GPL-2.0 or GPL-3.0</t>
-        </is>
-      </c>
-      <c r="F16" s="38" t="inlineStr">
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>Permissive</t>
+        </is>
+      </c>
+      <c r="G16" s="32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>Keep notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="23.85" customHeight="1" s="21">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>build-essential / g++</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>Debian packages in the mas builder stage</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>Compilers of the build stage, not shipped</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>Build tools (builder stage of a multi-stage Dockerfile)</t>
+        </is>
+      </c>
+      <c r="E17" s="25" t="inlineStr">
+        <is>
+          <t>GPL-3.0 with GCC Runtime Library Exception</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
         <is>
           <t>Strong copyleft</t>
         </is>
       </c>
-      <c r="G16" s="33" t="inlineStr">
-        <is>
-          <t>OK – conditions</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="inlineStr">
-        <is>
-          <t>Separate program = aggregation, Horus code unaffected. GPL texts in LICENSES/, written offer in THIRD_PARTY_NOTICES section 7, sources gathered by scripts/licences/fetch-gpl-sources.py (08/10). Replacing pdf2image+poppler with pypdfium2 would also remove GnuPG, which poppler pulls in.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="21">
-      <c r="A17" s="31" t="inlineStr">
-        <is>
-          <t>tesseract-ocr</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="inlineStr">
-        <is>
-          <t>Debian package in knowledge-store image</t>
-        </is>
-      </c>
-      <c r="C17" s="25" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
-      <c r="D17" s="25" t="inlineStr">
-        <is>
-          <t>Separate program via pytesseract</t>
-        </is>
-      </c>
-      <c r="E17" s="25" t="inlineStr">
-        <is>
-          <t>Apache-2.0</t>
-        </is>
-      </c>
-      <c r="F17" s="32" t="inlineStr">
-        <is>
-          <t>Permissive</t>
-        </is>
-      </c>
-      <c r="G17" s="32" t="inlineStr">
+      <c r="G17" s="42" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H17" s="25" t="inlineStr">
         <is>
-          <t>Keep notice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="23.85" customHeight="1" s="21">
-      <c r="A18" s="31" t="inlineStr">
-        <is>
-          <t>build-essential / g++</t>
-        </is>
-      </c>
-      <c r="B18" s="31" t="inlineStr">
-        <is>
-          <t>Debian packages in the mas builder stage</t>
-        </is>
-      </c>
-      <c r="C18" s="25" t="inlineStr">
-        <is>
-          <t>Compilers of the build stage, not shipped</t>
-        </is>
-      </c>
-      <c r="D18" s="25" t="inlineStr">
-        <is>
-          <t>Build tools (builder stage of a multi-stage Dockerfile)</t>
-        </is>
-      </c>
-      <c r="E18" s="25" t="inlineStr">
-        <is>
-          <t>GPL-3.0 with GCC Runtime Library Exception</t>
-        </is>
-      </c>
-      <c r="F18" s="38" t="inlineStr">
-        <is>
-          <t>Strong copyleft</t>
-        </is>
-      </c>
-      <c r="G18" s="42" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="inlineStr">
-        <is>
           <t>Not in the image since 08/10: the MAS Dockerfile is multi-stage and its final stage installs no system package.</t>
         </is>
       </c>
     </row>
+    <row r="18" s="21"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -63782,7 +63745,7 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>src/infra/docker-compose.yml (dev-tools profile)</t>
+          <t>src/infra/docker-compose.yml</t>
         </is>
       </c>
       <c r="E4" s="25" t="inlineStr">
@@ -63797,7 +63760,7 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>RedisInsight and pgAdmin moved to the Compose profile dev-tools; the installer never starts it and no longer checks their ports.</t>
+          <t>Removed from the Compose file on 08/10 (its connection was never set up); valkey-cli in the redis container does the same job. pgAdmin stays in the dev-tools profile.</t>
         </is>
       </c>
       <c r="H4" s="31" t="inlineStr">
@@ -63807,7 +63770,7 @@
       </c>
       <c r="I4" s="31" t="inlineStr">
         <is>
-          <t>Done (07/10)</t>
+          <t>Done (08/10)</t>
         </is>
       </c>
     </row>

</xml_diff>